<commit_message>
Finalize analysis dashboard and executive deliverables
</commit_message>
<xml_diff>
--- a/outputs/analysis/attribution_models.xlsx
+++ b/outputs/analysis/attribution_models.xlsx
@@ -14,13 +14,15 @@
     <sheet name="Linear" sheetId="5" r:id="rId5"/>
     <sheet name="Time-Decay" sheetId="6" r:id="rId6"/>
     <sheet name="Model Comparison" sheetId="7" r:id="rId7"/>
+    <sheet name="Coverage and Scope" sheetId="8" r:id="rId8"/>
+    <sheet name="Method Definitions" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="76">
   <si>
     <t>channel</t>
   </si>
@@ -112,91 +114,142 @@
     <t>Marketing Sourced</t>
   </si>
   <si>
-    <t>$3,577,649</t>
-  </si>
-  <si>
-    <t>$2,664,782</t>
-  </si>
-  <si>
-    <t>$250,366</t>
-  </si>
-  <si>
-    <t>$557,743</t>
-  </si>
-  <si>
-    <t>$220,479</t>
-  </si>
-  <si>
-    <t>$51,984</t>
+    <t>$3,625,867</t>
+  </si>
+  <si>
+    <t>$2,716,112</t>
+  </si>
+  <si>
+    <t>$562,646</t>
+  </si>
+  <si>
+    <t>$224,743</t>
   </si>
   <si>
     <t>Marketing Influenced</t>
   </si>
   <si>
-    <t>$4,027,620</t>
-  </si>
-  <si>
-    <t>$1,982,244</t>
-  </si>
-  <si>
-    <t>$482,934</t>
+    <t>$4,055,120</t>
+  </si>
+  <si>
+    <t>$2,286,860</t>
   </si>
   <si>
     <t>$583,987</t>
   </si>
   <si>
-    <t>$136,181</t>
-  </si>
-  <si>
-    <t>$110,038</t>
+    <t>$203,401</t>
   </si>
   <si>
     <t>First-Touch</t>
   </si>
   <si>
-    <t>$3,270,957</t>
-  </si>
-  <si>
-    <t>$3,026,104</t>
-  </si>
-  <si>
-    <t>$195,736</t>
-  </si>
-  <si>
-    <t>$342,837</t>
+    <t>$3,231,875</t>
+  </si>
+  <si>
+    <t>$3,110,104</t>
+  </si>
+  <si>
+    <t>$303,755</t>
   </si>
   <si>
     <t>$483,634</t>
   </si>
   <si>
-    <t>$3,736</t>
-  </si>
-  <si>
     <t>Last-Touch</t>
   </si>
   <si>
     <t>Linear</t>
   </si>
   <si>
-    <t>$3,507,545</t>
-  </si>
-  <si>
-    <t>$2,831,696</t>
-  </si>
-  <si>
-    <t>$153,557</t>
-  </si>
-  <si>
-    <t>$337,001</t>
-  </si>
-  <si>
-    <t>$479,775</t>
-  </si>
-  <si>
-    <t>$13,430</t>
+    <t>$3,312,179</t>
+  </si>
+  <si>
+    <t>$3,029,801</t>
+  </si>
+  <si>
+    <t>$285,822</t>
+  </si>
+  <si>
+    <t>$501,567</t>
   </si>
   <si>
     <t>Time-Decay</t>
+  </si>
+  <si>
+    <t>lookback_days</t>
+  </si>
+  <si>
+    <t>all_opportunities</t>
+  </si>
+  <si>
+    <t>eligible_domain_date_amount</t>
+  </si>
+  <si>
+    <t>linked_opportunities</t>
+  </si>
+  <si>
+    <t>linked_share_of_all_opportunities</t>
+  </si>
+  <si>
+    <t>all_won_opportunities</t>
+  </si>
+  <si>
+    <t>eligible_won_opportunities</t>
+  </si>
+  <si>
+    <t>linked_won_opportunities</t>
+  </si>
+  <si>
+    <t>linked_share_of_won_opportunities</t>
+  </si>
+  <si>
+    <t>linked_pipeline</t>
+  </si>
+  <si>
+    <t>linked_won_revenue</t>
+  </si>
+  <si>
+    <t>touchpoint_grain</t>
+  </si>
+  <si>
+    <t>web_rule</t>
+  </si>
+  <si>
+    <t>one account-channel presence per ISO week</t>
+  </si>
+  <si>
+    <t>blank-UTM web sessions excluded from marketing attribution</t>
+  </si>
+  <si>
+    <t>Assumption</t>
+  </si>
+  <si>
+    <t>Definition</t>
+  </si>
+  <si>
+    <t>Lookback window</t>
+  </si>
+  <si>
+    <t>Touchpoint normalization</t>
+  </si>
+  <si>
+    <t>Web classification</t>
+  </si>
+  <si>
+    <t>Interpretation</t>
+  </si>
+  <si>
+    <t>Marketing touchpoint occurred 0-365 days before opportunity creation.</t>
+  </si>
+  <si>
+    <t>One account-channel presence per ISO week; source-row frequency is not treated as cross-channel importance.</t>
+  </si>
+  <si>
+    <t>Sessions without a non-blank UTM source or campaign are excluded from marketing attribution.</t>
+  </si>
+  <si>
+    <t>Attribution describes observed journey association and credit allocation; it does not estimate incremental causal lift.</t>
   </si>
 </sst>
 </file>
@@ -708,7 +761,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -736,13 +789,13 @@
         <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2">
         <v>594</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -753,30 +806,13 @@
         <v>31</v>
       </c>
       <c r="C3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3">
+        <v>360</v>
+      </c>
+      <c r="E3" t="s">
         <v>34</v>
-      </c>
-      <c r="D3">
-        <v>362</v>
-      </c>
-      <c r="E3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4">
-        <v>45</v>
-      </c>
-      <c r="E4" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -786,7 +822,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -811,16 +847,16 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2">
+        <v>509</v>
+      </c>
+      <c r="D2" t="s">
         <v>37</v>
       </c>
-      <c r="C2">
-        <v>506</v>
-      </c>
-      <c r="D2" t="s">
-        <v>40</v>
-      </c>
       <c r="E2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -828,33 +864,16 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3">
+        <v>186</v>
+      </c>
+      <c r="D3" t="s">
         <v>38</v>
       </c>
-      <c r="C3">
-        <v>159</v>
-      </c>
-      <c r="D3" t="s">
-        <v>41</v>
-      </c>
       <c r="E3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
         <v>39</v>
-      </c>
-      <c r="C4">
-        <v>43</v>
-      </c>
-      <c r="D4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -864,7 +883,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -889,16 +908,16 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2">
+        <v>268</v>
+      </c>
+      <c r="D2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E2" t="s">
         <v>44</v>
-      </c>
-      <c r="C2">
-        <v>269</v>
-      </c>
-      <c r="D2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -906,33 +925,16 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C3">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -942,7 +944,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -970,13 +972,13 @@
         <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2">
         <v>594</v>
       </c>
       <c r="E2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -987,30 +989,13 @@
         <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D3">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4">
         <v>45</v>
-      </c>
-      <c r="E4" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1020,7 +1005,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1045,16 +1030,16 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D2">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="E2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1062,33 +1047,16 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="D3">
         <v>594</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D4">
-        <v>45</v>
-      </c>
-      <c r="E4" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1106,22 +1074,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D1" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
         <v>29</v>
       </c>
       <c r="G1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -1152,22 +1120,22 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>1982243.82</v>
+        <v>2286859.82</v>
       </c>
       <c r="C3">
-        <v>3270957.4</v>
+        <v>3231875.4</v>
       </c>
       <c r="D3">
-        <v>2664782.2</v>
+        <v>2716112.2</v>
       </c>
       <c r="E3">
-        <v>2664782.2</v>
+        <v>2716112.2</v>
       </c>
       <c r="F3">
         <v>89016</v>
       </c>
       <c r="G3">
-        <v>3507544.762609037</v>
+        <v>3312178.694695475</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1198,22 +1166,22 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>4027619.54</v>
+        <v>4055119.54</v>
       </c>
       <c r="C5">
-        <v>3026103.96</v>
+        <v>3110103.96</v>
       </c>
       <c r="D5">
-        <v>3577648.66</v>
+        <v>3625867.16</v>
       </c>
       <c r="E5">
-        <v>3577648.66</v>
+        <v>3625867.16</v>
       </c>
       <c r="F5">
         <v>91226.5</v>
       </c>
       <c r="G5">
-        <v>2831696.06769459</v>
+        <v>3029800.665304525</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1290,22 +1258,22 @@
         <v>6</v>
       </c>
       <c r="B9">
-        <v>482934</v>
+        <v>0</v>
       </c>
       <c r="C9">
-        <v>195736</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>250366.5</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>250366.5</v>
+        <v>0</v>
       </c>
       <c r="F9">
         <v>1100230</v>
       </c>
       <c r="G9">
-        <v>153556.5296963728</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -1329,6 +1297,148 @@
       </c>
       <c r="G10">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H1" t="s">
+        <v>58</v>
+      </c>
+      <c r="I1" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1" t="s">
+        <v>60</v>
+      </c>
+      <c r="K1" t="s">
+        <v>61</v>
+      </c>
+      <c r="L1" t="s">
+        <v>62</v>
+      </c>
+      <c r="M1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2">
+        <v>365</v>
+      </c>
+      <c r="B2">
+        <v>3288</v>
+      </c>
+      <c r="C2">
+        <v>3166</v>
+      </c>
+      <c r="D2">
+        <v>695</v>
+      </c>
+      <c r="E2">
+        <v>0.211374695863747</v>
+      </c>
+      <c r="F2">
+        <v>1073</v>
+      </c>
+      <c r="G2">
+        <v>1056</v>
+      </c>
+      <c r="H2">
+        <v>126</v>
+      </c>
+      <c r="I2">
+        <v>0.1174277726001864</v>
+      </c>
+      <c r="J2">
+        <v>6341979.359999999</v>
+      </c>
+      <c r="K2">
+        <v>787388.5700000001</v>
+      </c>
+      <c r="L2" t="s">
+        <v>64</v>
+      </c>
+      <c r="M2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ship content-preserving revenue command center dashboard
</commit_message>
<xml_diff>
--- a/outputs/analysis/attribution_models.xlsx
+++ b/outputs/analysis/attribution_models.xlsx
@@ -15,14 +15,15 @@
     <sheet name="Time-Decay" sheetId="6" r:id="rId6"/>
     <sheet name="Model Comparison" sheetId="7" r:id="rId7"/>
     <sheet name="Coverage and Scope" sheetId="8" r:id="rId8"/>
-    <sheet name="Method Definitions" sheetId="9" r:id="rId9"/>
+    <sheet name="Lookback Sensitivity" sheetId="9" r:id="rId9"/>
+    <sheet name="Method Definitions" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="76">
   <si>
     <t>channel</t>
   </si>
@@ -759,6 +760,56 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
@@ -1398,47 +1449,212 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="B1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B5" t="s">
-        <v>75</v>
+        <v>52</v>
+      </c>
+      <c r="C1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H1" t="s">
+        <v>58</v>
+      </c>
+      <c r="I1" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1" t="s">
+        <v>60</v>
+      </c>
+      <c r="K1" t="s">
+        <v>61</v>
+      </c>
+      <c r="L1" t="s">
+        <v>62</v>
+      </c>
+      <c r="M1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2">
+        <v>30</v>
+      </c>
+      <c r="B2">
+        <v>3288</v>
+      </c>
+      <c r="C2">
+        <v>3166</v>
+      </c>
+      <c r="D2">
+        <v>431</v>
+      </c>
+      <c r="E2">
+        <v>0.1310827250608272</v>
+      </c>
+      <c r="F2">
+        <v>1073</v>
+      </c>
+      <c r="G2">
+        <v>1056</v>
+      </c>
+      <c r="H2">
+        <v>65</v>
+      </c>
+      <c r="I2">
+        <v>0.06057781919850885</v>
+      </c>
+      <c r="J2">
+        <v>3995089.25</v>
+      </c>
+      <c r="K2">
+        <v>553783</v>
+      </c>
+      <c r="L2" t="s">
+        <v>64</v>
+      </c>
+      <c r="M2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3">
+        <v>90</v>
+      </c>
+      <c r="B3">
+        <v>3288</v>
+      </c>
+      <c r="C3">
+        <v>3166</v>
+      </c>
+      <c r="D3">
+        <v>593</v>
+      </c>
+      <c r="E3">
+        <v>0.180352798053528</v>
+      </c>
+      <c r="F3">
+        <v>1073</v>
+      </c>
+      <c r="G3">
+        <v>1056</v>
+      </c>
+      <c r="H3">
+        <v>101</v>
+      </c>
+      <c r="I3">
+        <v>0.09412861136999068</v>
+      </c>
+      <c r="J3">
+        <v>5674641.189999999</v>
+      </c>
+      <c r="K3">
+        <v>754341.3300000001</v>
+      </c>
+      <c r="L3" t="s">
+        <v>64</v>
+      </c>
+      <c r="M3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4">
+        <v>180</v>
+      </c>
+      <c r="B4">
+        <v>3288</v>
+      </c>
+      <c r="C4">
+        <v>3166</v>
+      </c>
+      <c r="D4">
+        <v>664</v>
+      </c>
+      <c r="E4">
+        <v>0.2019464720194647</v>
+      </c>
+      <c r="F4">
+        <v>1073</v>
+      </c>
+      <c r="G4">
+        <v>1056</v>
+      </c>
+      <c r="H4">
+        <v>118</v>
+      </c>
+      <c r="I4">
+        <v>0.1099720410065238</v>
+      </c>
+      <c r="J4">
+        <v>6199104.02</v>
+      </c>
+      <c r="K4">
+        <v>785815.23</v>
+      </c>
+      <c r="L4" t="s">
+        <v>64</v>
+      </c>
+      <c r="M4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5">
+        <v>365</v>
+      </c>
+      <c r="B5">
+        <v>3288</v>
+      </c>
+      <c r="C5">
+        <v>3166</v>
+      </c>
+      <c r="D5">
+        <v>695</v>
+      </c>
+      <c r="E5">
+        <v>0.211374695863747</v>
+      </c>
+      <c r="F5">
+        <v>1073</v>
+      </c>
+      <c r="G5">
+        <v>1056</v>
+      </c>
+      <c r="H5">
+        <v>126</v>
+      </c>
+      <c r="I5">
+        <v>0.1174277726001864</v>
+      </c>
+      <c r="J5">
+        <v>6341979.359999999</v>
+      </c>
+      <c r="K5">
+        <v>787388.5700000001</v>
+      </c>
+      <c r="L5" t="s">
+        <v>64</v>
+      </c>
+      <c r="M5" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>